<commit_message>
fix(burger-joint-checklists-en): ronda 1 de la revisión adversarial — 2 MAYOR + 12 menor aplicados
Boil-out mensual y aceite según TPM (no cambio mensual), queso americano, picada por encima del pollo crudo,
lectura de la make line, sonda con ice-point diario, utensilios cada 4 h (4-602.11(C)), trampa de grasa,
mínimos de inventario en formatos de compra US. Landing alineada. 5 hermanos idénticos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Via: Claude Code
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/burger-joint-checklist-templates/01-burger-joint-opening-closing-checklists.xlsx
+++ b/astro-site/public/dl/burger-joint-checklist-templates/01-burger-joint-opening-closing-checklists.xlsx
@@ -1408,9 +1408,9 @@
       <c r="A26" s="29" t="n">
         <v>19</v>
       </c>
-      <c r="B26" s="30" t="inlineStr">
-        <is>
-          <t>Slice cheese: cheddar, gouda, blue cheese, Swiss</t>
+      <c r="B26" s="34" t="inlineStr">
+        <is>
+          <t>Slice cheese: American, cheddar, gouda, blue cheese, Swiss</t>
         </is>
       </c>
       <c r="C26" s="27" t="inlineStr">
@@ -2560,7 +2560,7 @@
       </c>
       <c r="B6" s="33" t="inlineStr">
         <is>
-          <t>Store leftover beef in the walk-in: raw ground beef covered, date-marked, 41 °F or below, bottom shelf below ready-to-eat food (FDA 3-302.11)</t>
+          <t>Store leftover beef in the walk-in: raw ground beef covered, date-marked, 41 °F or below, below ready-to-eat food and above any raw chicken (FDA 3-302.11)</t>
         </is>
       </c>
       <c r="C6" s="27" t="inlineStr">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="B13" s="34" t="inlineStr">
         <is>
-          <t>Turn the fryer off after service and let the oil cool; the hood stays on meanwhile</t>
+          <t>Turn the fryer off after service; the hood stays on until the fryer and griddle have cooled</t>
         </is>
       </c>
       <c r="C13" s="27" t="inlineStr">
@@ -2762,7 +2762,7 @@
       </c>
       <c r="B14" s="33" t="inlineStr">
         <is>
-          <t>Filter or change the oil as the fryer manufacturer says (many have built-in hot filtering, others need to cool first); heat-resistant gloves, apron and goggles</t>
+          <t>Filter the oil every night as the fryer manufacturer says (built-in filtration usually runs with the oil still hot, right after service; a portable filter only once it has cooled to what the manual allows) and change it when the TPM tester says; heat-resistant gloves, apron and goggles</t>
         </is>
       </c>
       <c r="C14" s="27" t="inlineStr">

</xml_diff>